<commit_message>
Modification place entête documents et rajout de "SCAF DE" pour Longevelle.
</commit_message>
<xml_diff>
--- a/Documents/Classements/Classements_2310.xlsx
+++ b/Documents/Classements/Classements_2310.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WpfProject\Gestcom\Documents\Classements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF54326B-077E-4669-A736-A3AABCF17B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3EAE7DC-6FCD-41D3-BAA4-F4750FAAEB93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4128" yWindow="3396" windowWidth="17280" windowHeight="8964" firstSheet="4" activeTab="5" xr2:uid="{6053974A-3F34-40E8-94A7-4F82EB2C7DF3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="4" activeTab="5" xr2:uid="{6053974A-3F34-40E8-94A7-4F82EB2C7DF3}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -1033,7 +1033,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEACEF65-78A5-466F-9AD3-AF3EDA89E9C5}">
-  <dimension ref="A10:G37"/>
+  <dimension ref="A7:G37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="13.77734375" style="1" customWidth="1"/>
@@ -1044,23 +1044,23 @@
     <col min="7" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
+    <row r="7" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D8" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D9" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
     <row r="10" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D10" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D11" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D12" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="13" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D13" s="1" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>